<commit_message>
chore(data-release): publish site data 2026-10-23 11:19:15 UTC
</commit_message>
<xml_diff>
--- a/countries/de/2026-2029.xlsx
+++ b/countries/de/2026-2029.xlsx
@@ -1624,13 +1624,13 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O8" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="R8" t="n">
-        <v>0.09444760691164239</v>
+        <v>0.09564314623963786</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -5368,13 +5368,13 @@
         </is>
       </c>
       <c r="N34" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O34" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="R34" t="n">
-        <v>0.1829175171833074</v>
+        <v>0.1841130565113029</v>
       </c>
       <c r="U34" t="inlineStr">
         <is>
@@ -7528,13 +7528,13 @@
         </is>
       </c>
       <c r="N49" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="O49" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="R49" t="n">
-        <v>0.2642141914869996</v>
+        <v>0.2654097308149951</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -15304,13 +15304,13 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="O103" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R103" t="n">
-        <v>0.381377045630556</v>
+        <v>0.3825725849585515</v>
       </c>
       <c r="U103" t="inlineStr">
         <is>
@@ -19480,13 +19480,13 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O132" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R132" t="n">
-        <v>0.01554201126394116</v>
+        <v>0.01673755059193663</v>
       </c>
       <c r="U132" t="inlineStr">
         <is>
@@ -21640,13 +21640,13 @@
         </is>
       </c>
       <c r="N147" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O147" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R147" t="n">
-        <v>0.08727437094366955</v>
+        <v>0.08846991027166504</v>
       </c>
       <c r="U147" t="inlineStr">
         <is>
@@ -35032,13 +35032,13 @@
         </is>
       </c>
       <c r="N240" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="O240" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="R240" t="n">
-        <v>0.2713874274549725</v>
+        <v>0.270191888126977</v>
       </c>
       <c r="U240" t="inlineStr">
         <is>
@@ -39064,13 +39064,13 @@
         </is>
       </c>
       <c r="N268" t="n">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="O268" t="n">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="R268" t="n">
-        <v>0.5045175964140898</v>
+        <v>0.5057131357420852</v>
       </c>
       <c r="U268" t="inlineStr">
         <is>
@@ -43528,13 +43528,13 @@
         </is>
       </c>
       <c r="N299" t="n">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="O299" t="n">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="R299" t="n">
-        <v>1.761029430137332</v>
+        <v>1.762224969465328</v>
       </c>
       <c r="U299" t="inlineStr">
         <is>
@@ -45400,13 +45400,13 @@
         </is>
       </c>
       <c r="N312" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="O312" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="R312" t="n">
-        <v>0.4578915626222663</v>
+        <v>0.4590871019502618</v>
       </c>
       <c r="U312" t="inlineStr">
         <is>
@@ -47272,13 +47272,13 @@
         </is>
       </c>
       <c r="N325" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O325" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R325" t="n">
-        <v>0.01912862924792757</v>
+        <v>0.02032416857592305</v>
       </c>
       <c r="U325" t="inlineStr">
         <is>
@@ -47704,13 +47704,13 @@
         </is>
       </c>
       <c r="N328" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O328" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="R328" t="n">
-        <v>0.2797562027509408</v>
+        <v>0.2785606634229453</v>
       </c>
       <c r="U328" t="inlineStr">
         <is>
@@ -48568,13 +48568,13 @@
         </is>
       </c>
       <c r="N334" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O334" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="R334" t="n">
-        <v>0.3682261130226058</v>
+        <v>0.3694216523506013</v>
       </c>
       <c r="U334" t="inlineStr">
         <is>
@@ -50152,13 +50152,13 @@
         </is>
       </c>
       <c r="N345" t="n">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="O345" t="n">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="R345" t="n">
-        <v>1.655821969273731</v>
+        <v>1.657017508601726</v>
       </c>
       <c r="U345" t="inlineStr">
         <is>
@@ -51880,13 +51880,13 @@
         </is>
       </c>
       <c r="N357" t="n">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="O357" t="n">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="R357" t="n">
-        <v>0.4734335738862075</v>
+        <v>0.4758246525421984</v>
       </c>
       <c r="U357" t="inlineStr">
         <is>
@@ -52024,13 +52024,13 @@
         </is>
       </c>
       <c r="N358" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O358" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="R358" t="n">
-        <v>0.2211747756791626</v>
+        <v>0.222370315007158</v>
       </c>
       <c r="U358" t="inlineStr">
         <is>
@@ -53896,13 +53896,13 @@
         </is>
       </c>
       <c r="N371" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O371" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="R371" t="n">
-        <v>0.05379926975979631</v>
+        <v>0.05499480908779177</v>
       </c>
       <c r="U371" t="inlineStr">
         <is>
@@ -54040,13 +54040,13 @@
         </is>
       </c>
       <c r="N372" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O372" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R372" t="n">
-        <v>0.3204045399027869</v>
+        <v>0.3192090005747914</v>
       </c>
       <c r="U372" t="inlineStr">
         <is>
@@ -54184,13 +54184,13 @@
         </is>
       </c>
       <c r="N373" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O373" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="R373" t="n">
-        <v>0.1518334946554251</v>
+        <v>0.1506379553274297</v>
       </c>
       <c r="U373" t="inlineStr">
         <is>
@@ -56776,13 +56776,13 @@
         </is>
       </c>
       <c r="N391" t="n">
-        <v>1254</v>
+        <v>1257</v>
       </c>
       <c r="O391" t="n">
-        <v>1254</v>
+        <v>1257</v>
       </c>
       <c r="R391" t="n">
-        <v>1.499206317306324</v>
+        <v>1.50279293529031</v>
       </c>
       <c r="U391" t="inlineStr">
         <is>
@@ -57352,13 +57352,13 @@
         </is>
       </c>
       <c r="N395" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O395" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R395" t="n">
-        <v>0.01075985395195926</v>
+        <v>0.01195539327995473</v>
       </c>
       <c r="U395" t="inlineStr">
         <is>
@@ -57784,13 +57784,13 @@
         </is>
       </c>
       <c r="N398" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O398" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="R398" t="n">
-        <v>0.1291182474235111</v>
+        <v>0.1303137867515066</v>
       </c>
       <c r="U398" t="inlineStr">
         <is>
@@ -60952,13 +60952,13 @@
         </is>
       </c>
       <c r="N420" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O420" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="R420" t="n">
-        <v>0.2964937533428774</v>
+        <v>0.2976892926708729</v>
       </c>
       <c r="U420" t="inlineStr">
         <is>
@@ -61672,13 +61672,13 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O425" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="R425" t="n">
-        <v>0.05858142707177819</v>
+        <v>0.05977696639977367</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
@@ -61816,13 +61816,13 @@
         </is>
       </c>
       <c r="N426" t="n">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="O426" t="n">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="R426" t="n">
-        <v>0.4531094053102844</v>
+        <v>0.4543049446382799</v>
       </c>
       <c r="U426" t="inlineStr">
         <is>
@@ -62968,13 +62968,13 @@
         </is>
       </c>
       <c r="N434" t="n">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="O434" t="n">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="R434" t="n">
-        <v>0.3299688545267507</v>
+        <v>0.3287733151987552</v>
       </c>
       <c r="U434" t="inlineStr">
         <is>
@@ -63112,13 +63112,13 @@
         </is>
       </c>
       <c r="N435" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O435" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R435" t="n">
-        <v>0.04184387647984157</v>
+        <v>0.04303941580783704</v>
       </c>
       <c r="U435" t="inlineStr">
         <is>
@@ -63400,13 +63400,13 @@
         </is>
       </c>
       <c r="N437" t="n">
-        <v>1177</v>
+        <v>1187</v>
       </c>
       <c r="O437" t="n">
-        <v>1177</v>
+        <v>1187</v>
       </c>
       <c r="R437" t="n">
-        <v>1.407149789050672</v>
+        <v>1.419105182330627</v>
       </c>
       <c r="U437" t="inlineStr">
         <is>
@@ -63688,13 +63688,13 @@
         </is>
       </c>
       <c r="N439" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="O439" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="R439" t="n">
-        <v>0.07651451699171029</v>
+        <v>0.07890559564770125</v>
       </c>
       <c r="U439" t="inlineStr">
         <is>
@@ -65128,13 +65128,13 @@
         </is>
       </c>
       <c r="N449" t="n">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="O449" t="n">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="R449" t="n">
-        <v>0.3945279782385062</v>
+        <v>0.3981145962224927</v>
       </c>
       <c r="U449" t="inlineStr">
         <is>
@@ -65272,13 +65272,13 @@
         </is>
       </c>
       <c r="N450" t="n">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="O450" t="n">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="R450" t="n">
-        <v>0.202046146431235</v>
+        <v>0.2056327644152214</v>
       </c>
       <c r="U450" t="inlineStr">
         <is>
@@ -66280,13 +66280,13 @@
         </is>
       </c>
       <c r="N457" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O457" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="R457" t="n">
-        <v>0.2199792363511671</v>
+        <v>0.2211747756791626</v>
       </c>
       <c r="U457" t="inlineStr">
         <is>
@@ -67288,13 +67288,13 @@
         </is>
       </c>
       <c r="N464" t="n">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="O464" t="n">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="R464" t="n">
-        <v>0.3192090005747914</v>
+        <v>0.3168179219188005</v>
       </c>
       <c r="U464" t="inlineStr">
         <is>
@@ -67576,13 +67576,13 @@
         </is>
       </c>
       <c r="N466" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="O466" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="R466" t="n">
-        <v>0.1422691800314613</v>
+        <v>0.1434647193594568</v>
       </c>
       <c r="U466" t="inlineStr">
         <is>
@@ -67864,13 +67864,13 @@
         </is>
       </c>
       <c r="N468" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="O468" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="R468" t="n">
-        <v>0.06216804505576462</v>
+        <v>0.06455912371175557</v>
       </c>
       <c r="U468" t="inlineStr">
         <is>
@@ -68008,13 +68008,13 @@
         </is>
       </c>
       <c r="N469" t="n">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="O469" t="n">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="R469" t="n">
-        <v>0.5308194616299902</v>
+        <v>0.5391882369259585</v>
       </c>
       <c r="U469" t="inlineStr">
         <is>
@@ -69160,13 +69160,13 @@
         </is>
       </c>
       <c r="N477" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O477" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="R477" t="n">
-        <v>0.2905160567029</v>
+        <v>0.2917115960308955</v>
       </c>
       <c r="U477" t="inlineStr">
         <is>
@@ -69448,13 +69448,13 @@
         </is>
       </c>
       <c r="N479" t="n">
-        <v>1049</v>
+        <v>1085</v>
       </c>
       <c r="O479" t="n">
-        <v>1049</v>
+        <v>1085</v>
       </c>
       <c r="R479" t="n">
-        <v>1.254120755067252</v>
+        <v>1.297160170875089</v>
       </c>
       <c r="U479" t="inlineStr">
         <is>
@@ -69736,13 +69736,13 @@
         </is>
       </c>
       <c r="N481" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="O481" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="R481" t="n">
-        <v>0.07053682035173293</v>
+        <v>0.07173235967972839</v>
       </c>
       <c r="U481" t="inlineStr">
         <is>
@@ -70024,13 +70024,13 @@
         </is>
       </c>
       <c r="N483" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O483" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="R483" t="n">
-        <v>0.1123806968315745</v>
+        <v>0.11357623615957</v>
       </c>
       <c r="U483" t="inlineStr">
         <is>
@@ -70312,13 +70312,13 @@
         </is>
       </c>
       <c r="N485" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O485" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R485" t="n">
-        <v>0.06814574169574199</v>
+        <v>0.06934128102373746</v>
       </c>
       <c r="U485" t="inlineStr">
         <is>
@@ -70600,13 +70600,13 @@
         </is>
       </c>
       <c r="N487" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="O487" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="R487" t="n">
-        <v>0.247476640895063</v>
+        <v>0.2498677195510539</v>
       </c>
       <c r="U487" t="inlineStr">
         <is>
@@ -71032,13 +71032,13 @@
         </is>
       </c>
       <c r="N490" t="n">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="O490" t="n">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="R490" t="n">
-        <v>0.3371420904947235</v>
+        <v>0.3502930231026737</v>
       </c>
       <c r="U490" t="inlineStr">
         <is>
@@ -71176,13 +71176,13 @@
         </is>
       </c>
       <c r="N491" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="O491" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="R491" t="n">
-        <v>0.2104149217272033</v>
+        <v>0.2128060003831942</v>
       </c>
       <c r="U491" t="inlineStr">
         <is>
@@ -71896,13 +71896,13 @@
         </is>
       </c>
       <c r="N496" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O496" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R496" t="n">
-        <v>0.08846991027166504</v>
+        <v>0.0896654495996605</v>
       </c>
       <c r="U496" t="inlineStr">
         <is>
@@ -72040,13 +72040,13 @@
         </is>
       </c>
       <c r="N497" t="n">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="O497" t="n">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="R497" t="n">
-        <v>0.1876996744952893</v>
+        <v>0.1924818318072712</v>
       </c>
       <c r="U497" t="inlineStr">
         <is>
@@ -72328,13 +72328,13 @@
         </is>
       </c>
       <c r="N499" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O499" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="R499" t="n">
-        <v>0.2462811015670675</v>
+        <v>0.245085562239072</v>
       </c>
       <c r="U499" t="inlineStr">
         <is>
@@ -72472,13 +72472,13 @@
         </is>
       </c>
       <c r="N500" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O500" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R500" t="n">
-        <v>0.002391078655990946</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U500" t="inlineStr">
         <is>
@@ -72760,13 +72760,13 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="O502" t="n">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="R502" t="n">
-        <v>1.097505103099845</v>
+        <v>1.09870064242784</v>
       </c>
       <c r="U502" t="inlineStr">
         <is>
@@ -72904,13 +72904,13 @@
         </is>
       </c>
       <c r="N503" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O503" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R503" t="n">
-        <v>0.04184387647984157</v>
+        <v>0.04303941580783704</v>
       </c>
       <c r="U503" t="inlineStr">
         <is>
@@ -73048,13 +73048,13 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="O504" t="n">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="R504" t="n">
-        <v>0.2952982140148819</v>
+        <v>0.2917115960308955</v>
       </c>
       <c r="U504" t="inlineStr">
         <is>
@@ -73192,13 +73192,13 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O505" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="R505" t="n">
-        <v>0.1542245733114161</v>
+        <v>0.1554201126394116</v>
       </c>
       <c r="U505" t="inlineStr">
         <is>
@@ -73336,13 +73336,13 @@
         </is>
       </c>
       <c r="N506" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="O506" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="R506" t="n">
-        <v>0.09086098892765598</v>
+        <v>0.09683868556763335</v>
       </c>
       <c r="U506" t="inlineStr">
         <is>
@@ -73624,13 +73624,13 @@
         </is>
       </c>
       <c r="N508" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="O508" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="R508" t="n">
-        <v>0.06097250572776914</v>
+        <v>0.06336358438376009</v>
       </c>
       <c r="U508" t="inlineStr">
         <is>
@@ -73768,13 +73768,13 @@
         </is>
       </c>
       <c r="N509" t="n">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="O509" t="n">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="R509" t="n">
-        <v>0.4363718547183478</v>
+        <v>0.4555004839662754</v>
       </c>
       <c r="U509" t="inlineStr">
         <is>
@@ -74344,13 +74344,13 @@
         </is>
       </c>
       <c r="N513" t="n">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="O513" t="n">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="R513" t="n">
-        <v>0.6563510910695148</v>
+        <v>0.6611332483814968</v>
       </c>
       <c r="U513" t="inlineStr">
         <is>
@@ -74488,13 +74488,13 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O514" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R514" t="n">
-        <v>0.004782157311981893</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U514" t="inlineStr">
         <is>
@@ -74632,13 +74632,13 @@
         </is>
       </c>
       <c r="N515" t="n">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="O515" t="n">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="R515" t="n">
-        <v>0.3000803713268638</v>
+        <v>0.3024714499828547</v>
       </c>
       <c r="U515" t="inlineStr">
         <is>
@@ -74776,13 +74776,13 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O516" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="R516" t="n">
-        <v>0.02510632588790494</v>
+        <v>0.02749740454389589</v>
       </c>
       <c r="U516" t="inlineStr">
         <is>
@@ -74920,13 +74920,13 @@
         </is>
       </c>
       <c r="N517" t="n">
-        <v>726</v>
+        <v>780</v>
       </c>
       <c r="O517" t="n">
-        <v>726</v>
+        <v>780</v>
       </c>
       <c r="R517" t="n">
-        <v>0.8679615521247137</v>
+        <v>0.9325206758364692</v>
       </c>
       <c r="U517" t="inlineStr">
         <is>
@@ -75064,13 +75064,13 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="O518" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="R518" t="n">
-        <v>0.04543049446382799</v>
+        <v>0.05021265177580988</v>
       </c>
       <c r="U518" t="inlineStr">
         <is>
@@ -75208,13 +75208,13 @@
         </is>
       </c>
       <c r="N519" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="O519" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="R519" t="n">
-        <v>0.04423495513583252</v>
+        <v>0.05140819110380536</v>
       </c>
       <c r="U519" t="inlineStr">
         <is>
@@ -75640,13 +75640,13 @@
         </is>
       </c>
       <c r="N522" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="O522" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="R522" t="n">
-        <v>0.1052074608636017</v>
+        <v>0.111185157503579</v>
       </c>
       <c r="U522" t="inlineStr">
         <is>
@@ -75784,13 +75784,13 @@
         </is>
       </c>
       <c r="N523" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O523" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R523" t="n">
-        <v>0.1960684497912576</v>
+        <v>0.1972639891192531</v>
       </c>
       <c r="U523" t="inlineStr">
         <is>
@@ -76216,13 +76216,13 @@
         </is>
       </c>
       <c r="N526" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="O526" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="R526" t="n">
-        <v>0.2151970790391852</v>
+        <v>0.2175881576951762</v>
       </c>
       <c r="U526" t="inlineStr">
         <is>
@@ -76648,13 +76648,13 @@
         </is>
       </c>
       <c r="N529" t="n">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="O529" t="n">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="R529" t="n">
-        <v>0.2761695847669544</v>
+        <v>0.2917115960308955</v>
       </c>
       <c r="U529" t="inlineStr">
         <is>
@@ -76792,13 +76792,13 @@
         </is>
       </c>
       <c r="N530" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="O530" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="R530" t="n">
-        <v>0.1530290339834206</v>
+        <v>0.1625933486073844</v>
       </c>
       <c r="U530" t="inlineStr">
         <is>
@@ -77080,13 +77080,13 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O532" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R532" t="n">
-        <v>0.001195539327995473</v>
+        <v>0.002391078655990946</v>
       </c>
       <c r="U532" t="inlineStr">
         <is>
@@ -77224,13 +77224,13 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O533" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R533" t="n">
-        <v>0.04543049446382799</v>
+        <v>0.04423495513583252</v>
       </c>
       <c r="U533" t="inlineStr">
         <is>
@@ -77368,13 +77368,13 @@
         </is>
       </c>
       <c r="N534" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O534" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="R534" t="n">
-        <v>0.04303941580783704</v>
+        <v>0.04543049446382799</v>
       </c>
       <c r="U534" t="inlineStr">
         <is>
@@ -77512,13 +77512,13 @@
         </is>
       </c>
       <c r="N535" t="n">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="O535" t="n">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="R535" t="n">
-        <v>0.1757442812153346</v>
+        <v>0.1829175171833074</v>
       </c>
       <c r="U535" t="inlineStr">
         <is>
@@ -77656,13 +77656,13 @@
         </is>
       </c>
       <c r="N536" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O536" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R536" t="n">
-        <v>0.007173235967972841</v>
+        <v>0.009564314623963786</v>
       </c>
       <c r="U536" t="inlineStr">
         <is>
@@ -77800,13 +77800,13 @@
         </is>
       </c>
       <c r="N537" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="O537" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="R537" t="n">
-        <v>0.2534543375350404</v>
+        <v>0.2558454161910313</v>
       </c>
       <c r="U537" t="inlineStr">
         <is>
@@ -77944,13 +77944,13 @@
         </is>
       </c>
       <c r="N538" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O538" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R538" t="n">
-        <v>0.02151970790391852</v>
+        <v>0.022715247231914</v>
       </c>
       <c r="U538" t="inlineStr">
         <is>
@@ -78199,7 +78199,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>61198</v>
+        <v>61441</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore: update partitioned data downloads
</commit_message>
<xml_diff>
--- a/countries/de/2026-2029.xlsx
+++ b/countries/de/2026-2029.xlsx
@@ -1624,13 +1624,13 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O8" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="R8" t="n">
-        <v>0.09564314623963786</v>
+        <v>0.09683868556763335</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -17176,13 +17176,13 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>1838</v>
+        <v>1839</v>
       </c>
       <c r="O116" t="n">
-        <v>1838</v>
+        <v>1839</v>
       </c>
       <c r="R116" t="n">
-        <v>2.19740128485568</v>
+        <v>2.198596824183675</v>
       </c>
       <c r="U116" t="inlineStr">
         <is>
@@ -20056,13 +20056,13 @@
         </is>
       </c>
       <c r="N136" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O136" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R136" t="n">
-        <v>0.06097250572776914</v>
+        <v>0.06216804505576462</v>
       </c>
       <c r="U136" t="inlineStr">
         <is>
@@ -23656,13 +23656,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="O161" t="n">
-        <v>1650</v>
+        <v>1651</v>
       </c>
       <c r="R161" t="n">
-        <v>1.972639891192531</v>
+        <v>1.973835430520526</v>
       </c>
       <c r="U161" t="inlineStr">
         <is>
@@ -27976,13 +27976,13 @@
         </is>
       </c>
       <c r="N191" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="O191" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="R191" t="n">
-        <v>0.2331301689591173</v>
+        <v>0.2343257082871128</v>
       </c>
       <c r="U191" t="inlineStr">
         <is>
@@ -35752,13 +35752,13 @@
         </is>
       </c>
       <c r="N245" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="O245" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="R245" t="n">
-        <v>0.08249221363168767</v>
+        <v>0.0812966743036922</v>
       </c>
       <c r="U245" t="inlineStr">
         <is>
@@ -37336,13 +37336,13 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>1450</v>
+        <v>1452</v>
       </c>
       <c r="O256" t="n">
-        <v>1450</v>
+        <v>1452</v>
       </c>
       <c r="R256" t="n">
-        <v>1.733532025593436</v>
+        <v>1.735923104249427</v>
       </c>
       <c r="U256" t="inlineStr">
         <is>
@@ -38632,13 +38632,13 @@
         </is>
       </c>
       <c r="N265" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="O265" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="R265" t="n">
-        <v>0.4387629333743387</v>
+        <v>0.4399584727023342</v>
       </c>
       <c r="U265" t="inlineStr">
         <is>
@@ -41224,13 +41224,13 @@
         </is>
       </c>
       <c r="N283" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O283" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="R283" t="n">
-        <v>0.04782157311981893</v>
+        <v>0.04901711244781441</v>
       </c>
       <c r="U283" t="inlineStr">
         <is>
@@ -41368,13 +41368,13 @@
         </is>
       </c>
       <c r="N284" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O284" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="R284" t="n">
-        <v>0.2785606634229453</v>
+        <v>0.2797562027509408</v>
       </c>
       <c r="U284" t="inlineStr">
         <is>
@@ -43528,13 +43528,13 @@
         </is>
       </c>
       <c r="N299" t="n">
-        <v>1474</v>
+        <v>1476</v>
       </c>
       <c r="O299" t="n">
-        <v>1474</v>
+        <v>1476</v>
       </c>
       <c r="R299" t="n">
-        <v>1.762224969465328</v>
+        <v>1.764616048121319</v>
       </c>
       <c r="U299" t="inlineStr">
         <is>
@@ -43672,13 +43672,13 @@
         </is>
       </c>
       <c r="N300" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O300" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="R300" t="n">
-        <v>0.08249221363168767</v>
+        <v>0.08368775295968314</v>
       </c>
       <c r="U300" t="inlineStr">
         <is>
@@ -45400,13 +45400,13 @@
         </is>
       </c>
       <c r="N312" t="n">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="O312" t="n">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="R312" t="n">
-        <v>0.4590871019502618</v>
+        <v>0.4602826412782573</v>
       </c>
       <c r="U312" t="inlineStr">
         <is>
@@ -45544,13 +45544,13 @@
         </is>
       </c>
       <c r="N313" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O313" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R313" t="n">
-        <v>0.2582364948470223</v>
+        <v>0.2594320341750177</v>
       </c>
       <c r="U313" t="inlineStr">
         <is>
@@ -47272,13 +47272,13 @@
         </is>
       </c>
       <c r="N325" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O325" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R325" t="n">
-        <v>0.02032416857592305</v>
+        <v>0.02151970790391852</v>
       </c>
       <c r="U325" t="inlineStr">
         <is>
@@ -48424,13 +48424,13 @@
         </is>
       </c>
       <c r="N333" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="O333" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R333" t="n">
-        <v>0.07890559564770125</v>
+        <v>0.08010113497569672</v>
       </c>
       <c r="U333" t="inlineStr">
         <is>
@@ -52024,13 +52024,13 @@
         </is>
       </c>
       <c r="N358" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O358" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="R358" t="n">
-        <v>0.222370315007158</v>
+        <v>0.2235658543351535</v>
       </c>
       <c r="U358" t="inlineStr">
         <is>
@@ -54040,13 +54040,13 @@
         </is>
       </c>
       <c r="N372" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="O372" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="R372" t="n">
-        <v>0.3192090005747914</v>
+        <v>0.3180134612467959</v>
       </c>
       <c r="U372" t="inlineStr">
         <is>
@@ -54184,13 +54184,13 @@
         </is>
       </c>
       <c r="N373" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="O373" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="R373" t="n">
-        <v>0.1506379553274297</v>
+        <v>0.1530290339834206</v>
       </c>
       <c r="U373" t="inlineStr">
         <is>
@@ -54328,13 +54328,13 @@
         </is>
       </c>
       <c r="N374" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O374" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R374" t="n">
-        <v>0.1398781013754704</v>
+        <v>0.1410736407034659</v>
       </c>
       <c r="U374" t="inlineStr">
         <is>
@@ -54904,13 +54904,13 @@
         </is>
       </c>
       <c r="N378" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="O378" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="R378" t="n">
-        <v>0.4076789108464564</v>
+        <v>0.4088744501744519</v>
       </c>
       <c r="U378" t="inlineStr">
         <is>
@@ -56776,13 +56776,13 @@
         </is>
       </c>
       <c r="N391" t="n">
-        <v>1257</v>
+        <v>1261</v>
       </c>
       <c r="O391" t="n">
-        <v>1257</v>
+        <v>1261</v>
       </c>
       <c r="R391" t="n">
-        <v>1.50279293529031</v>
+        <v>1.507575092602292</v>
       </c>
       <c r="U391" t="inlineStr">
         <is>
@@ -56920,13 +56920,13 @@
         </is>
       </c>
       <c r="N392" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O392" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R392" t="n">
-        <v>0.07771005631970578</v>
+        <v>0.07890559564770125</v>
       </c>
       <c r="U392" t="inlineStr">
         <is>
@@ -57064,13 +57064,13 @@
         </is>
       </c>
       <c r="N393" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O393" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="R393" t="n">
-        <v>0.0896654495996605</v>
+        <v>0.09086098892765598</v>
       </c>
       <c r="U393" t="inlineStr">
         <is>
@@ -59944,13 +59944,13 @@
         </is>
       </c>
       <c r="N413" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="O413" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="R413" t="n">
-        <v>0.2534543375350404</v>
+        <v>0.2558454161910313</v>
       </c>
       <c r="U413" t="inlineStr">
         <is>
@@ -61672,13 +61672,13 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="O425" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="R425" t="n">
-        <v>0.05977696639977367</v>
+        <v>0.06216804505576462</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
@@ -61816,13 +61816,13 @@
         </is>
       </c>
       <c r="N426" t="n">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="O426" t="n">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="R426" t="n">
-        <v>0.4543049446382799</v>
+        <v>0.4566960232942708</v>
       </c>
       <c r="U426" t="inlineStr">
         <is>
@@ -62248,13 +62248,13 @@
         </is>
       </c>
       <c r="N429" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O429" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R429" t="n">
-        <v>0.00358661798398642</v>
+        <v>0.004782157311981893</v>
       </c>
       <c r="U429" t="inlineStr">
         <is>
@@ -63400,13 +63400,13 @@
         </is>
       </c>
       <c r="N437" t="n">
-        <v>1187</v>
+        <v>1191</v>
       </c>
       <c r="O437" t="n">
-        <v>1187</v>
+        <v>1191</v>
       </c>
       <c r="R437" t="n">
-        <v>1.419105182330627</v>
+        <v>1.423887339642609</v>
       </c>
       <c r="U437" t="inlineStr">
         <is>
@@ -64696,13 +64696,13 @@
         </is>
       </c>
       <c r="N446" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O446" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="R446" t="n">
-        <v>0.2905160567029</v>
+        <v>0.2917115960308955</v>
       </c>
       <c r="U446" t="inlineStr">
         <is>
@@ -65272,13 +65272,13 @@
         </is>
       </c>
       <c r="N450" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O450" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="R450" t="n">
-        <v>0.2056327644152214</v>
+        <v>0.2068283037432169</v>
       </c>
       <c r="U450" t="inlineStr">
         <is>
@@ -66280,13 +66280,13 @@
         </is>
       </c>
       <c r="N457" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="O457" t="n">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="R457" t="n">
-        <v>0.2211747756791626</v>
+        <v>0.2235658543351535</v>
       </c>
       <c r="U457" t="inlineStr">
         <is>
@@ -67000,13 +67000,13 @@
         </is>
       </c>
       <c r="N462" t="n">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="O462" t="n">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="R462" t="n">
-        <v>1.030554900732098</v>
+        <v>1.031750440060094</v>
       </c>
       <c r="U462" t="inlineStr">
         <is>
@@ -67288,13 +67288,13 @@
         </is>
       </c>
       <c r="N464" t="n">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="O464" t="n">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="R464" t="n">
-        <v>0.3168179219188005</v>
+        <v>0.313231303934814</v>
       </c>
       <c r="U464" t="inlineStr">
         <is>
@@ -67576,13 +67576,13 @@
         </is>
       </c>
       <c r="N466" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="O466" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="R466" t="n">
-        <v>0.1434647193594568</v>
+        <v>0.1446602586874523</v>
       </c>
       <c r="U466" t="inlineStr">
         <is>
@@ -67864,13 +67864,13 @@
         </is>
       </c>
       <c r="N468" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="O468" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="R468" t="n">
-        <v>0.06455912371175557</v>
+        <v>0.06695020236774651</v>
       </c>
       <c r="U468" t="inlineStr">
         <is>
@@ -68008,13 +68008,13 @@
         </is>
       </c>
       <c r="N469" t="n">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="O469" t="n">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="R469" t="n">
-        <v>0.5391882369259585</v>
+        <v>0.540383776253954</v>
       </c>
       <c r="U469" t="inlineStr">
         <is>
@@ -68440,13 +68440,13 @@
         </is>
       </c>
       <c r="N472" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O472" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R472" t="n">
-        <v>0.001195539327995473</v>
+        <v>0.007173235967972841</v>
       </c>
       <c r="U472" t="inlineStr">
         <is>
@@ -68872,13 +68872,13 @@
         </is>
       </c>
       <c r="N475" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O475" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R475" t="n">
-        <v>0.005977696639977366</v>
+        <v>0.004782157311981893</v>
       </c>
       <c r="U475" t="inlineStr">
         <is>
@@ -69448,13 +69448,13 @@
         </is>
       </c>
       <c r="N479" t="n">
-        <v>1085</v>
+        <v>1105</v>
       </c>
       <c r="O479" t="n">
-        <v>1085</v>
+        <v>1105</v>
       </c>
       <c r="R479" t="n">
-        <v>1.297160170875089</v>
+        <v>1.321070957434998</v>
       </c>
       <c r="U479" t="inlineStr">
         <is>
@@ -69592,13 +69592,13 @@
         </is>
       </c>
       <c r="N480" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="O480" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="R480" t="n">
-        <v>0.07053682035173293</v>
+        <v>0.07173235967972839</v>
       </c>
       <c r="U480" t="inlineStr">
         <is>
@@ -70024,13 +70024,13 @@
         </is>
       </c>
       <c r="N483" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="O483" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="R483" t="n">
-        <v>0.11357623615957</v>
+        <v>0.1183583934715519</v>
       </c>
       <c r="U483" t="inlineStr">
         <is>
@@ -70168,13 +70168,13 @@
         </is>
       </c>
       <c r="N484" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O484" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="R484" t="n">
-        <v>0.1948729104632622</v>
+        <v>0.1960684497912576</v>
       </c>
       <c r="U484" t="inlineStr">
         <is>
@@ -71032,13 +71032,13 @@
         </is>
       </c>
       <c r="N490" t="n">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="O490" t="n">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="R490" t="n">
-        <v>0.3502930231026737</v>
+        <v>0.3598573377266375</v>
       </c>
       <c r="U490" t="inlineStr">
         <is>
@@ -71176,13 +71176,13 @@
         </is>
       </c>
       <c r="N491" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="O491" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="R491" t="n">
-        <v>0.2128060003831942</v>
+        <v>0.2140015397111897</v>
       </c>
       <c r="U491" t="inlineStr">
         <is>
@@ -71291,17 +71291,17 @@
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>D124</t>
+          <t>D123</t>
         </is>
       </c>
       <c r="I492" t="inlineStr">
         <is>
-          <t>Typhoid fever</t>
+          <t>Tularemia</t>
         </is>
       </c>
       <c r="J492" t="inlineStr">
         <is>
-          <t>伤寒</t>
+          <t>土拉菌病</t>
         </is>
       </c>
       <c r="K492" t="inlineStr">
@@ -71320,17 +71320,17 @@
         </is>
       </c>
       <c r="N492" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O492" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R492" t="n">
-        <v>0.00358661798398642</v>
+        <v>0.005977696639977366</v>
       </c>
       <c r="U492" t="inlineStr">
         <is>
-          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
+          <t>HOLD_DE_b849fa63b7ae6fabb95bdf916fe8</t>
         </is>
       </c>
       <c r="AA492" t="inlineStr">
@@ -71350,7 +71350,7 @@
       </c>
       <c r="AS492" t="inlineStr">
         <is>
-          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
+          <t>HOLD_DE_b849fa63b7ae6fabb95bdf916fe8</t>
         </is>
       </c>
       <c r="AT492" t="n">
@@ -71435,17 +71435,17 @@
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>D126</t>
+          <t>D124</t>
         </is>
       </c>
       <c r="I493" t="inlineStr">
         <is>
-          <t>Vibriosis</t>
+          <t>Typhoid fever</t>
         </is>
       </c>
       <c r="J493" t="inlineStr">
         <is>
-          <t>弧菌病</t>
+          <t>伤寒</t>
         </is>
       </c>
       <c r="K493" t="inlineStr">
@@ -71464,17 +71464,17 @@
         </is>
       </c>
       <c r="N493" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O493" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R493" t="n">
-        <v>0.002391078655990946</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U493" t="inlineStr">
         <is>
-          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
+          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
         </is>
       </c>
       <c r="AA493" t="inlineStr">
@@ -71494,7 +71494,7 @@
       </c>
       <c r="AS493" t="inlineStr">
         <is>
-          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
+          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
         </is>
       </c>
       <c r="AT493" t="n">
@@ -71579,22 +71579,22 @@
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>D128</t>
+          <t>D126</t>
         </is>
       </c>
       <c r="I494" t="inlineStr">
         <is>
-          <t>West Nile virus</t>
+          <t>Vibriosis</t>
         </is>
       </c>
       <c r="J494" t="inlineStr">
         <is>
-          <t>西尼罗病毒</t>
+          <t>弧菌病</t>
         </is>
       </c>
       <c r="K494" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L494" t="inlineStr">
@@ -71608,17 +71608,17 @@
         </is>
       </c>
       <c r="N494" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O494" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R494" t="n">
-        <v>0.00358661798398642</v>
+        <v>0.002391078655990946</v>
       </c>
       <c r="U494" t="inlineStr">
         <is>
-          <t>HOLD_DE_bbdd653bfa640555b27f82fd1353</t>
+          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
         </is>
       </c>
       <c r="AA494" t="inlineStr">
@@ -71638,7 +71638,7 @@
       </c>
       <c r="AS494" t="inlineStr">
         <is>
-          <t>HOLD_DE_bbdd653bfa640555b27f82fd1353</t>
+          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
         </is>
       </c>
       <c r="AT494" t="n">
@@ -71723,17 +71723,17 @@
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>D142</t>
+          <t>D128</t>
         </is>
       </c>
       <c r="I495" t="inlineStr">
         <is>
-          <t>Respiratory syncytial virus infection (RSV)</t>
+          <t>West Nile virus</t>
         </is>
       </c>
       <c r="J495" t="inlineStr">
         <is>
-          <t>呼吸道合胞病毒感染</t>
+          <t>西尼罗病毒</t>
         </is>
       </c>
       <c r="K495" t="inlineStr">
@@ -71752,17 +71752,17 @@
         </is>
       </c>
       <c r="N495" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="O495" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="R495" t="n">
-        <v>0.03825725849585514</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U495" t="inlineStr">
         <is>
-          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
+          <t>HOLD_DE_bbdd653bfa640555b27f82fd1353</t>
         </is>
       </c>
       <c r="AA495" t="inlineStr">
@@ -71782,7 +71782,7 @@
       </c>
       <c r="AS495" t="inlineStr">
         <is>
-          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
+          <t>HOLD_DE_bbdd653bfa640555b27f82fd1353</t>
         </is>
       </c>
       <c r="AT495" t="n">
@@ -71867,22 +71867,22 @@
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>D155</t>
+          <t>D142</t>
         </is>
       </c>
       <c r="I496" t="inlineStr">
         <is>
-          <t>Yersiniosis</t>
+          <t>Respiratory syncytial virus infection (RSV)</t>
         </is>
       </c>
       <c r="J496" t="inlineStr">
         <is>
-          <t>耶尔森菌病</t>
+          <t>呼吸道合胞病毒感染</t>
         </is>
       </c>
       <c r="K496" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L496" t="inlineStr">
@@ -71896,17 +71896,17 @@
         </is>
       </c>
       <c r="N496" t="n">
-        <v>75</v>
+        <v>32</v>
       </c>
       <c r="O496" t="n">
-        <v>75</v>
+        <v>32</v>
       </c>
       <c r="R496" t="n">
-        <v>0.0896654495996605</v>
+        <v>0.03825725849585514</v>
       </c>
       <c r="U496" t="inlineStr">
         <is>
-          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
+          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
         </is>
       </c>
       <c r="AA496" t="inlineStr">
@@ -71926,7 +71926,7 @@
       </c>
       <c r="AS496" t="inlineStr">
         <is>
-          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
+          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
         </is>
       </c>
       <c r="AT496" t="n">
@@ -72011,22 +72011,22 @@
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>D199</t>
+          <t>D155</t>
         </is>
       </c>
       <c r="I497" t="inlineStr">
         <is>
-          <t>Rotavirus infection</t>
+          <t>Yersiniosis</t>
         </is>
       </c>
       <c r="J497" t="inlineStr">
         <is>
-          <t>轮状病毒感染</t>
+          <t>耶尔森菌病</t>
         </is>
       </c>
       <c r="K497" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L497" t="inlineStr">
@@ -72040,17 +72040,17 @@
         </is>
       </c>
       <c r="N497" t="n">
-        <v>161</v>
+        <v>77</v>
       </c>
       <c r="O497" t="n">
-        <v>161</v>
+        <v>77</v>
       </c>
       <c r="R497" t="n">
-        <v>0.1924818318072712</v>
+        <v>0.09205652825565144</v>
       </c>
       <c r="U497" t="inlineStr">
         <is>
-          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
+          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
         </is>
       </c>
       <c r="AA497" t="inlineStr">
@@ -72070,7 +72070,7 @@
       </c>
       <c r="AS497" t="inlineStr">
         <is>
-          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
+          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
         </is>
       </c>
       <c r="AT497" t="n">
@@ -72155,17 +72155,17 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>D205</t>
+          <t>D199</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
         <is>
-          <t>Tick-borne encephalitis</t>
+          <t>Rotavirus infection</t>
         </is>
       </c>
       <c r="J498" t="inlineStr">
         <is>
-          <t>蜱传脑炎</t>
+          <t>轮状病毒感染</t>
         </is>
       </c>
       <c r="K498" t="inlineStr">
@@ -72184,17 +72184,17 @@
         </is>
       </c>
       <c r="N498" t="n">
-        <v>15</v>
+        <v>163</v>
       </c>
       <c r="O498" t="n">
-        <v>15</v>
+        <v>163</v>
       </c>
       <c r="R498" t="n">
-        <v>0.0179330899199321</v>
+        <v>0.1948729104632622</v>
       </c>
       <c r="U498" t="inlineStr">
         <is>
-          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
+          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
         </is>
       </c>
       <c r="AA498" t="inlineStr">
@@ -72214,7 +72214,7 @@
       </c>
       <c r="AS498" t="inlineStr">
         <is>
-          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
+          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
         </is>
       </c>
       <c r="AT498" t="n">
@@ -72299,22 +72299,22 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>D227</t>
+          <t>D205</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
         <is>
-          <t>Carbapenem-resistant Enterobacterales infection</t>
+          <t>Tick-borne encephalitis</t>
         </is>
       </c>
       <c r="J499" t="inlineStr">
         <is>
-          <t>碳青霉烯耐药肠杆菌目细菌感染</t>
+          <t>蜱传脑炎</t>
         </is>
       </c>
       <c r="K499" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L499" t="inlineStr">
@@ -72328,17 +72328,17 @@
         </is>
       </c>
       <c r="N499" t="n">
-        <v>205</v>
+        <v>15</v>
       </c>
       <c r="O499" t="n">
-        <v>205</v>
+        <v>15</v>
       </c>
       <c r="R499" t="n">
-        <v>0.245085562239072</v>
+        <v>0.0179330899199321</v>
       </c>
       <c r="U499" t="inlineStr">
         <is>
-          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
+          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
         </is>
       </c>
       <c r="AA499" t="inlineStr">
@@ -72358,7 +72358,7 @@
       </c>
       <c r="AS499" t="inlineStr">
         <is>
-          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
+          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
         </is>
       </c>
       <c r="AT499" t="n">
@@ -72443,17 +72443,17 @@
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>D234</t>
+          <t>D227</t>
         </is>
       </c>
       <c r="I500" t="inlineStr">
         <is>
-          <t>Paratyphoid fever</t>
+          <t>Carbapenem-resistant Enterobacterales infection</t>
         </is>
       </c>
       <c r="J500" t="inlineStr">
         <is>
-          <t>副伤寒</t>
+          <t>碳青霉烯耐药肠杆菌目细菌感染</t>
         </is>
       </c>
       <c r="K500" t="inlineStr">
@@ -72472,17 +72472,17 @@
         </is>
       </c>
       <c r="N500" t="n">
-        <v>3</v>
+        <v>205</v>
       </c>
       <c r="O500" t="n">
-        <v>3</v>
+        <v>205</v>
       </c>
       <c r="R500" t="n">
-        <v>0.00358661798398642</v>
+        <v>0.245085562239072</v>
       </c>
       <c r="U500" t="inlineStr">
         <is>
-          <t>HOLD_DE_ad719d2726b8d2f22f4647a5f85a</t>
+          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
         </is>
       </c>
       <c r="AA500" t="inlineStr">
@@ -72502,7 +72502,7 @@
       </c>
       <c r="AS500" t="inlineStr">
         <is>
-          <t>HOLD_DE_ad719d2726b8d2f22f4647a5f85a</t>
+          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
         </is>
       </c>
       <c r="AT500" t="n">
@@ -72587,17 +72587,17 @@
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>D236</t>
+          <t>D234</t>
         </is>
       </c>
       <c r="I501" t="inlineStr">
         <is>
-          <t>Methicillin-resistant Staphylococcus aureus (MRSA) surveillance</t>
+          <t>Paratyphoid fever</t>
         </is>
       </c>
       <c r="J501" t="inlineStr">
         <is>
-          <t>耐甲氧西林金黄色葡萄球菌（MRSA）监测</t>
+          <t>副伤寒</t>
         </is>
       </c>
       <c r="K501" t="inlineStr">
@@ -72616,17 +72616,17 @@
         </is>
       </c>
       <c r="N501" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="O501" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="R501" t="n">
-        <v>0.02032416857592305</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U501" t="inlineStr">
         <is>
-          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
+          <t>HOLD_DE_ad719d2726b8d2f22f4647a5f85a</t>
         </is>
       </c>
       <c r="AA501" t="inlineStr">
@@ -72646,7 +72646,7 @@
       </c>
       <c r="AS501" t="inlineStr">
         <is>
-          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
+          <t>HOLD_DE_ad719d2726b8d2f22f4647a5f85a</t>
         </is>
       </c>
       <c r="AT501" t="n">
@@ -72731,27 +72731,27 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>D004</t>
+          <t>D236</t>
         </is>
       </c>
       <c r="I502" t="inlineStr">
         <is>
-          <t>COVID-19</t>
+          <t>Methicillin-resistant Staphylococcus aureus (MRSA) surveillance</t>
         </is>
       </c>
       <c r="J502" t="inlineStr">
         <is>
-          <t>新型冠状病毒感染</t>
+          <t>耐甲氧西林金黄色葡萄球菌（MRSA）监测</t>
         </is>
       </c>
       <c r="K502" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L502" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="M502" t="inlineStr">
@@ -72760,17 +72760,17 @@
         </is>
       </c>
       <c r="N502" t="n">
-        <v>919</v>
+        <v>17</v>
       </c>
       <c r="O502" t="n">
-        <v>919</v>
+        <v>17</v>
       </c>
       <c r="R502" t="n">
-        <v>1.09870064242784</v>
+        <v>0.02032416857592305</v>
       </c>
       <c r="U502" t="inlineStr">
         <is>
-          <t>HOLD_DE_254d1e1533c2313cd38064c471e8</t>
+          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
         </is>
       </c>
       <c r="AA502" t="inlineStr">
@@ -72790,7 +72790,7 @@
       </c>
       <c r="AS502" t="inlineStr">
         <is>
-          <t>HOLD_DE_254d1e1533c2313cd38064c471e8</t>
+          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
         </is>
       </c>
       <c r="AT502" t="n">
@@ -72875,17 +72875,17 @@
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>D007</t>
+          <t>D004</t>
         </is>
       </c>
       <c r="I503" t="inlineStr">
         <is>
-          <t>Hepatitis A</t>
+          <t>COVID-19</t>
         </is>
       </c>
       <c r="J503" t="inlineStr">
         <is>
-          <t>甲型肝炎</t>
+          <t>新型冠状病毒感染</t>
         </is>
       </c>
       <c r="K503" t="inlineStr">
@@ -72904,17 +72904,17 @@
         </is>
       </c>
       <c r="N503" t="n">
-        <v>36</v>
+        <v>919</v>
       </c>
       <c r="O503" t="n">
-        <v>36</v>
+        <v>919</v>
       </c>
       <c r="R503" t="n">
-        <v>0.04303941580783704</v>
+        <v>1.09870064242784</v>
       </c>
       <c r="U503" t="inlineStr">
         <is>
-          <t>HOLD_DE_a24da742c3570a7186ddc81fe39d</t>
+          <t>HOLD_DE_254d1e1533c2313cd38064c471e8</t>
         </is>
       </c>
       <c r="AA503" t="inlineStr">
@@ -72934,7 +72934,7 @@
       </c>
       <c r="AS503" t="inlineStr">
         <is>
-          <t>HOLD_DE_a24da742c3570a7186ddc81fe39d</t>
+          <t>HOLD_DE_254d1e1533c2313cd38064c471e8</t>
         </is>
       </c>
       <c r="AT503" t="n">
@@ -73019,17 +73019,17 @@
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>D008</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I504" t="inlineStr">
         <is>
-          <t>Hepatitis B</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J504" t="inlineStr">
         <is>
-          <t>乙型肝炎</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K504" t="inlineStr">
@@ -73048,17 +73048,17 @@
         </is>
       </c>
       <c r="N504" t="n">
-        <v>244</v>
+        <v>37</v>
       </c>
       <c r="O504" t="n">
-        <v>244</v>
+        <v>37</v>
       </c>
       <c r="R504" t="n">
-        <v>0.2917115960308955</v>
+        <v>0.04423495513583252</v>
       </c>
       <c r="U504" t="inlineStr">
         <is>
-          <t>HOLD_DE_3fe4070a01910244ac558ce89feb</t>
+          <t>HOLD_DE_a24da742c3570a7186ddc81fe39d</t>
         </is>
       </c>
       <c r="AA504" t="inlineStr">
@@ -73078,7 +73078,7 @@
       </c>
       <c r="AS504" t="inlineStr">
         <is>
-          <t>HOLD_DE_3fe4070a01910244ac558ce89feb</t>
+          <t>HOLD_DE_a24da742c3570a7186ddc81fe39d</t>
         </is>
       </c>
       <c r="AT504" t="n">
@@ -73163,17 +73163,17 @@
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>D009</t>
+          <t>D008</t>
         </is>
       </c>
       <c r="I505" t="inlineStr">
         <is>
-          <t>Hepatitis C</t>
+          <t>Hepatitis B</t>
         </is>
       </c>
       <c r="J505" t="inlineStr">
         <is>
-          <t>丙型肝炎</t>
+          <t>乙型肝炎</t>
         </is>
       </c>
       <c r="K505" t="inlineStr">
@@ -73192,17 +73192,17 @@
         </is>
       </c>
       <c r="N505" t="n">
-        <v>130</v>
+        <v>242</v>
       </c>
       <c r="O505" t="n">
-        <v>130</v>
+        <v>242</v>
       </c>
       <c r="R505" t="n">
-        <v>0.1554201126394116</v>
+        <v>0.2893205173749046</v>
       </c>
       <c r="U505" t="inlineStr">
         <is>
-          <t>HOLD_DE_58b36fad94e3f55b6f553ce94f61</t>
+          <t>HOLD_DE_3fe4070a01910244ac558ce89feb</t>
         </is>
       </c>
       <c r="AA505" t="inlineStr">
@@ -73222,7 +73222,7 @@
       </c>
       <c r="AS505" t="inlineStr">
         <is>
-          <t>HOLD_DE_58b36fad94e3f55b6f553ce94f61</t>
+          <t>HOLD_DE_3fe4070a01910244ac558ce89feb</t>
         </is>
       </c>
       <c r="AT505" t="n">
@@ -73307,17 +73307,17 @@
       </c>
       <c r="H506" t="inlineStr">
         <is>
-          <t>D011</t>
+          <t>D009</t>
         </is>
       </c>
       <c r="I506" t="inlineStr">
         <is>
-          <t>Hepatitis E</t>
+          <t>Hepatitis C</t>
         </is>
       </c>
       <c r="J506" t="inlineStr">
         <is>
-          <t>戊型肝炎</t>
+          <t>丙型肝炎</t>
         </is>
       </c>
       <c r="K506" t="inlineStr">
@@ -73336,17 +73336,17 @@
         </is>
       </c>
       <c r="N506" t="n">
-        <v>81</v>
+        <v>130</v>
       </c>
       <c r="O506" t="n">
-        <v>81</v>
+        <v>130</v>
       </c>
       <c r="R506" t="n">
-        <v>0.09683868556763335</v>
+        <v>0.1554201126394116</v>
       </c>
       <c r="U506" t="inlineStr">
         <is>
-          <t>HOLD_DE_560e9fa27cdd32ad9a1d28cd0b0d</t>
+          <t>HOLD_DE_58b36fad94e3f55b6f553ce94f61</t>
         </is>
       </c>
       <c r="AA506" t="inlineStr">
@@ -73366,7 +73366,7 @@
       </c>
       <c r="AS506" t="inlineStr">
         <is>
-          <t>HOLD_DE_560e9fa27cdd32ad9a1d28cd0b0d</t>
+          <t>HOLD_DE_58b36fad94e3f55b6f553ce94f61</t>
         </is>
       </c>
       <c r="AT506" t="n">
@@ -73451,17 +73451,17 @@
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D011</t>
         </is>
       </c>
       <c r="I507" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Hepatitis E</t>
         </is>
       </c>
       <c r="J507" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>戊型肝炎</t>
         </is>
       </c>
       <c r="K507" t="inlineStr">
@@ -73480,17 +73480,17 @@
         </is>
       </c>
       <c r="N507" t="n">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="O507" t="n">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="R507" t="n">
-        <v>0.004782157311981893</v>
+        <v>0.1052074608636017</v>
       </c>
       <c r="U507" t="inlineStr">
         <is>
-          <t>HOLD_DE_67a8383c9171c23bf4f8d0335669</t>
+          <t>HOLD_DE_560e9fa27cdd32ad9a1d28cd0b0d</t>
         </is>
       </c>
       <c r="AA507" t="inlineStr">
@@ -73510,7 +73510,7 @@
       </c>
       <c r="AS507" t="inlineStr">
         <is>
-          <t>HOLD_DE_67a8383c9171c23bf4f8d0335669</t>
+          <t>HOLD_DE_560e9fa27cdd32ad9a1d28cd0b0d</t>
         </is>
       </c>
       <c r="AT507" t="n">
@@ -73595,22 +73595,22 @@
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>D025</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I508" t="inlineStr">
         <is>
-          <t>Tuberculosis</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J508" t="inlineStr">
         <is>
-          <t>肺结核</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K508" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L508" t="inlineStr">
@@ -73624,17 +73624,17 @@
         </is>
       </c>
       <c r="N508" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="O508" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="R508" t="n">
-        <v>0.06336358438376009</v>
+        <v>0.004782157311981893</v>
       </c>
       <c r="U508" t="inlineStr">
         <is>
-          <t>HOLD_DE_1b0737fcd510170ff45815c0d362</t>
+          <t>HOLD_DE_67a8383c9171c23bf4f8d0335669</t>
         </is>
       </c>
       <c r="AA508" t="inlineStr">
@@ -73654,7 +73654,7 @@
       </c>
       <c r="AS508" t="inlineStr">
         <is>
-          <t>HOLD_DE_1b0737fcd510170ff45815c0d362</t>
+          <t>HOLD_DE_67a8383c9171c23bf4f8d0335669</t>
         </is>
       </c>
       <c r="AT508" t="n">
@@ -73739,17 +73739,17 @@
       </c>
       <c r="H509" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D025</t>
         </is>
       </c>
       <c r="I509" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Tuberculosis</t>
         </is>
       </c>
       <c r="J509" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>肺结核</t>
         </is>
       </c>
       <c r="K509" t="inlineStr">
@@ -73768,17 +73768,17 @@
         </is>
       </c>
       <c r="N509" t="n">
-        <v>381</v>
+        <v>54</v>
       </c>
       <c r="O509" t="n">
-        <v>381</v>
+        <v>54</v>
       </c>
       <c r="R509" t="n">
-        <v>0.4555004839662754</v>
+        <v>0.06455912371175557</v>
       </c>
       <c r="U509" t="inlineStr">
         <is>
-          <t>HOLD_DE_b7116f22f4c269b49252863c2b1b</t>
+          <t>HOLD_DE_1b0737fcd510170ff45815c0d362</t>
         </is>
       </c>
       <c r="AA509" t="inlineStr">
@@ -73798,7 +73798,7 @@
       </c>
       <c r="AS509" t="inlineStr">
         <is>
-          <t>HOLD_DE_b7116f22f4c269b49252863c2b1b</t>
+          <t>HOLD_DE_1b0737fcd510170ff45815c0d362</t>
         </is>
       </c>
       <c r="AT509" t="n">
@@ -73883,17 +73883,17 @@
       </c>
       <c r="H510" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I510" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J510" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K510" t="inlineStr">
@@ -73912,17 +73912,17 @@
         </is>
       </c>
       <c r="N510" t="n">
-        <v>1</v>
+        <v>392</v>
       </c>
       <c r="O510" t="n">
-        <v>1</v>
+        <v>392</v>
       </c>
       <c r="R510" t="n">
-        <v>0.001195539327995473</v>
+        <v>0.4686514165742255</v>
       </c>
       <c r="U510" t="inlineStr">
         <is>
-          <t>HOLD_DE_cf73ff0499232520079e651b4d44</t>
+          <t>HOLD_DE_b7116f22f4c269b49252863c2b1b</t>
         </is>
       </c>
       <c r="AA510" t="inlineStr">
@@ -73942,7 +73942,7 @@
       </c>
       <c r="AS510" t="inlineStr">
         <is>
-          <t>HOLD_DE_cf73ff0499232520079e651b4d44</t>
+          <t>HOLD_DE_b7116f22f4c269b49252863c2b1b</t>
         </is>
       </c>
       <c r="AT510" t="n">
@@ -74027,17 +74027,17 @@
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>D031</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I511" t="inlineStr">
         <is>
-          <t>Scarlet fever</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J511" t="inlineStr">
         <is>
-          <t>猩红热</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K511" t="inlineStr">
@@ -74056,17 +74056,17 @@
         </is>
       </c>
       <c r="N511" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O511" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R511" t="n">
-        <v>0.004782157311981893</v>
+        <v>0.001195539327995473</v>
       </c>
       <c r="U511" t="inlineStr">
         <is>
-          <t>HOLD_DE_c4a11116520e85cee113bf27f857</t>
+          <t>HOLD_DE_cf73ff0499232520079e651b4d44</t>
         </is>
       </c>
       <c r="AA511" t="inlineStr">
@@ -74086,7 +74086,7 @@
       </c>
       <c r="AS511" t="inlineStr">
         <is>
-          <t>HOLD_DE_c4a11116520e85cee113bf27f857</t>
+          <t>HOLD_DE_cf73ff0499232520079e651b4d44</t>
         </is>
       </c>
       <c r="AT511" t="n">
@@ -74171,22 +74171,22 @@
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>D037</t>
+          <t>D031</t>
         </is>
       </c>
       <c r="I512" t="inlineStr">
         <is>
-          <t>Malaria</t>
+          <t>Scarlet fever</t>
         </is>
       </c>
       <c r="J512" t="inlineStr">
         <is>
-          <t>疟疾</t>
+          <t>猩红热</t>
         </is>
       </c>
       <c r="K512" t="inlineStr">
         <is>
-          <t>Parasitic</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L512" t="inlineStr">
@@ -74200,17 +74200,17 @@
         </is>
       </c>
       <c r="N512" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="O512" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="R512" t="n">
-        <v>0.01434647193594568</v>
+        <v>0.004782157311981893</v>
       </c>
       <c r="U512" t="inlineStr">
         <is>
-          <t>HOLD_DE_ad052d1085b7281c5a415cb1f8fe</t>
+          <t>HOLD_DE_c4a11116520e85cee113bf27f857</t>
         </is>
       </c>
       <c r="AA512" t="inlineStr">
@@ -74230,7 +74230,7 @@
       </c>
       <c r="AS512" t="inlineStr">
         <is>
-          <t>HOLD_DE_ad052d1085b7281c5a415cb1f8fe</t>
+          <t>HOLD_DE_c4a11116520e85cee113bf27f857</t>
         </is>
       </c>
       <c r="AT512" t="n">
@@ -74315,22 +74315,22 @@
       </c>
       <c r="H513" t="inlineStr">
         <is>
-          <t>D038</t>
+          <t>D035</t>
         </is>
       </c>
       <c r="I513" t="inlineStr">
         <is>
-          <t>Influenza</t>
+          <t>Leptospirosis</t>
         </is>
       </c>
       <c r="J513" t="inlineStr">
         <is>
-          <t>流行性感冒</t>
+          <t>钩端螺旋体病</t>
         </is>
       </c>
       <c r="K513" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L513" t="inlineStr">
@@ -74344,17 +74344,17 @@
         </is>
       </c>
       <c r="N513" t="n">
-        <v>553</v>
+        <v>4</v>
       </c>
       <c r="O513" t="n">
-        <v>553</v>
+        <v>4</v>
       </c>
       <c r="R513" t="n">
-        <v>0.6611332483814968</v>
+        <v>0.004782157311981893</v>
       </c>
       <c r="U513" t="inlineStr">
         <is>
-          <t>HOLD_DE_7f5db8a8b4bbb456aed459172dc8</t>
+          <t>HOLD_DE_74d512ad41eaf3e22d516cca8020</t>
         </is>
       </c>
       <c r="AA513" t="inlineStr">
@@ -74374,7 +74374,7 @@
       </c>
       <c r="AS513" t="inlineStr">
         <is>
-          <t>HOLD_DE_7f5db8a8b4bbb456aed459172dc8</t>
+          <t>HOLD_DE_74d512ad41eaf3e22d516cca8020</t>
         </is>
       </c>
       <c r="AT513" t="n">
@@ -74459,22 +74459,22 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>D039</t>
+          <t>D037</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
         <is>
-          <t>Mumps</t>
+          <t>Malaria</t>
         </is>
       </c>
       <c r="J514" t="inlineStr">
         <is>
-          <t>流行性腮腺炎</t>
+          <t>疟疾</t>
         </is>
       </c>
       <c r="K514" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Parasitic</t>
         </is>
       </c>
       <c r="L514" t="inlineStr">
@@ -74488,17 +74488,17 @@
         </is>
       </c>
       <c r="N514" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="O514" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="R514" t="n">
-        <v>0.00358661798398642</v>
+        <v>0.01434647193594568</v>
       </c>
       <c r="U514" t="inlineStr">
         <is>
-          <t>HOLD_DE_0bf12d70d32e8f6a2cc183cc1b99</t>
+          <t>HOLD_DE_ad052d1085b7281c5a415cb1f8fe</t>
         </is>
       </c>
       <c r="AA514" t="inlineStr">
@@ -74518,7 +74518,7 @@
       </c>
       <c r="AS514" t="inlineStr">
         <is>
-          <t>HOLD_DE_0bf12d70d32e8f6a2cc183cc1b99</t>
+          <t>HOLD_DE_ad052d1085b7281c5a415cb1f8fe</t>
         </is>
       </c>
       <c r="AT514" t="n">
@@ -74603,17 +74603,17 @@
       </c>
       <c r="H515" t="inlineStr">
         <is>
-          <t>D054</t>
+          <t>D038</t>
         </is>
       </c>
       <c r="I515" t="inlineStr">
         <is>
-          <t>Varicella</t>
+          <t>Influenza</t>
         </is>
       </c>
       <c r="J515" t="inlineStr">
         <is>
-          <t>水痘</t>
+          <t>流行性感冒</t>
         </is>
       </c>
       <c r="K515" t="inlineStr">
@@ -74632,17 +74632,17 @@
         </is>
       </c>
       <c r="N515" t="n">
-        <v>253</v>
+        <v>553</v>
       </c>
       <c r="O515" t="n">
-        <v>253</v>
+        <v>553</v>
       </c>
       <c r="R515" t="n">
-        <v>0.3024714499828547</v>
+        <v>0.6611332483814968</v>
       </c>
       <c r="U515" t="inlineStr">
         <is>
-          <t>HOLD_DE_05d6c78e659357672953aebf8f89</t>
+          <t>HOLD_DE_7f5db8a8b4bbb456aed459172dc8</t>
         </is>
       </c>
       <c r="AA515" t="inlineStr">
@@ -74662,7 +74662,7 @@
       </c>
       <c r="AS515" t="inlineStr">
         <is>
-          <t>HOLD_DE_05d6c78e659357672953aebf8f89</t>
+          <t>HOLD_DE_7f5db8a8b4bbb456aed459172dc8</t>
         </is>
       </c>
       <c r="AT515" t="n">
@@ -74747,17 +74747,17 @@
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>D065</t>
+          <t>D039</t>
         </is>
       </c>
       <c r="I516" t="inlineStr">
         <is>
-          <t>Monkeypox</t>
+          <t>Mumps</t>
         </is>
       </c>
       <c r="J516" t="inlineStr">
         <is>
-          <t>猴痘</t>
+          <t>流行性腮腺炎</t>
         </is>
       </c>
       <c r="K516" t="inlineStr">
@@ -74776,17 +74776,17 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="O516" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="R516" t="n">
-        <v>0.02749740454389589</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U516" t="inlineStr">
         <is>
-          <t>HOLD_DE_6d498fe2f8fff0e559a9778cf771</t>
+          <t>HOLD_DE_0bf12d70d32e8f6a2cc183cc1b99</t>
         </is>
       </c>
       <c r="AA516" t="inlineStr">
@@ -74806,7 +74806,7 @@
       </c>
       <c r="AS516" t="inlineStr">
         <is>
-          <t>HOLD_DE_6d498fe2f8fff0e559a9778cf771</t>
+          <t>HOLD_DE_0bf12d70d32e8f6a2cc183cc1b99</t>
         </is>
       </c>
       <c r="AT516" t="n">
@@ -74891,22 +74891,22 @@
       </c>
       <c r="H517" t="inlineStr">
         <is>
-          <t>D092</t>
+          <t>D054</t>
         </is>
       </c>
       <c r="I517" t="inlineStr">
         <is>
-          <t>Campylobacteriosis</t>
+          <t>Varicella</t>
         </is>
       </c>
       <c r="J517" t="inlineStr">
         <is>
-          <t>弯曲杆菌病</t>
+          <t>水痘</t>
         </is>
       </c>
       <c r="K517" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L517" t="inlineStr">
@@ -74920,17 +74920,17 @@
         </is>
       </c>
       <c r="N517" t="n">
-        <v>780</v>
+        <v>256</v>
       </c>
       <c r="O517" t="n">
-        <v>780</v>
+        <v>256</v>
       </c>
       <c r="R517" t="n">
-        <v>0.9325206758364692</v>
+        <v>0.3060580679668412</v>
       </c>
       <c r="U517" t="inlineStr">
         <is>
-          <t>HOLD_DE_bcf3ec79b1fa22e487fecbdd29cb</t>
+          <t>HOLD_DE_05d6c78e659357672953aebf8f89</t>
         </is>
       </c>
       <c r="AA517" t="inlineStr">
@@ -74950,7 +74950,7 @@
       </c>
       <c r="AS517" t="inlineStr">
         <is>
-          <t>HOLD_DE_bcf3ec79b1fa22e487fecbdd29cb</t>
+          <t>HOLD_DE_05d6c78e659357672953aebf8f89</t>
         </is>
       </c>
       <c r="AT517" t="n">
@@ -75035,22 +75035,22 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>D096</t>
+          <t>D065</t>
         </is>
       </c>
       <c r="I518" t="inlineStr">
         <is>
-          <t>Cryptosporidiosis</t>
+          <t>Monkeypox</t>
         </is>
       </c>
       <c r="J518" t="inlineStr">
         <is>
-          <t>隐孢子虫病</t>
+          <t>猴痘</t>
         </is>
       </c>
       <c r="K518" t="inlineStr">
         <is>
-          <t>Parasitic</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L518" t="inlineStr">
@@ -75064,17 +75064,17 @@
         </is>
       </c>
       <c r="N518" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="O518" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="R518" t="n">
-        <v>0.05021265177580988</v>
+        <v>0.02869294387189136</v>
       </c>
       <c r="U518" t="inlineStr">
         <is>
-          <t>HOLD_DE_141fbc63db3a3fc81063e7f242e6</t>
+          <t>HOLD_DE_6d498fe2f8fff0e559a9778cf771</t>
         </is>
       </c>
       <c r="AA518" t="inlineStr">
@@ -75094,7 +75094,7 @@
       </c>
       <c r="AS518" t="inlineStr">
         <is>
-          <t>HOLD_DE_141fbc63db3a3fc81063e7f242e6</t>
+          <t>HOLD_DE_6d498fe2f8fff0e559a9778cf771</t>
         </is>
       </c>
       <c r="AT518" t="n">
@@ -75179,22 +75179,22 @@
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>D099</t>
+          <t>D092</t>
         </is>
       </c>
       <c r="I519" t="inlineStr">
         <is>
-          <t>Giardiasis</t>
+          <t>Campylobacteriosis</t>
         </is>
       </c>
       <c r="J519" t="inlineStr">
         <is>
-          <t>贾第虫病</t>
+          <t>弯曲杆菌病</t>
         </is>
       </c>
       <c r="K519" t="inlineStr">
         <is>
-          <t>Parasitic</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L519" t="inlineStr">
@@ -75208,17 +75208,17 @@
         </is>
       </c>
       <c r="N519" t="n">
-        <v>43</v>
+        <v>829</v>
       </c>
       <c r="O519" t="n">
-        <v>43</v>
+        <v>829</v>
       </c>
       <c r="R519" t="n">
-        <v>0.05140819110380536</v>
+        <v>0.9911021029082474</v>
       </c>
       <c r="U519" t="inlineStr">
         <is>
-          <t>HOLD_DE_e5f12cc63c1550ced86113ed9668</t>
+          <t>HOLD_DE_bcf3ec79b1fa22e487fecbdd29cb</t>
         </is>
       </c>
       <c r="AA519" t="inlineStr">
@@ -75238,7 +75238,7 @@
       </c>
       <c r="AS519" t="inlineStr">
         <is>
-          <t>HOLD_DE_e5f12cc63c1550ced86113ed9668</t>
+          <t>HOLD_DE_bcf3ec79b1fa22e487fecbdd29cb</t>
         </is>
       </c>
       <c r="AT519" t="n">
@@ -75323,22 +75323,22 @@
       </c>
       <c r="H520" t="inlineStr">
         <is>
-          <t>D102</t>
+          <t>D096</t>
         </is>
       </c>
       <c r="I520" t="inlineStr">
         <is>
-          <t>Hantavirus infection</t>
+          <t>Cryptosporidiosis</t>
         </is>
       </c>
       <c r="J520" t="inlineStr">
         <is>
-          <t>汉坦病毒感染</t>
+          <t>隐孢子虫病</t>
         </is>
       </c>
       <c r="K520" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Parasitic</t>
         </is>
       </c>
       <c r="L520" t="inlineStr">
@@ -75352,17 +75352,17 @@
         </is>
       </c>
       <c r="N520" t="n">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="O520" t="n">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="R520" t="n">
-        <v>0.004782157311981893</v>
+        <v>0.05140819110380536</v>
       </c>
       <c r="U520" t="inlineStr">
         <is>
-          <t>HOLD_DE_5cd9254a79f73f7e76719209af51</t>
+          <t>HOLD_DE_141fbc63db3a3fc81063e7f242e6</t>
         </is>
       </c>
       <c r="AA520" t="inlineStr">
@@ -75382,7 +75382,7 @@
       </c>
       <c r="AS520" t="inlineStr">
         <is>
-          <t>HOLD_DE_5cd9254a79f73f7e76719209af51</t>
+          <t>HOLD_DE_141fbc63db3a3fc81063e7f242e6</t>
         </is>
       </c>
       <c r="AT520" t="n">
@@ -75467,22 +75467,22 @@
       </c>
       <c r="H521" t="inlineStr">
         <is>
-          <t>D103</t>
+          <t>D099</t>
         </is>
       </c>
       <c r="I521" t="inlineStr">
         <is>
-          <t>Hemolytic uremic syndrome</t>
+          <t>Giardiasis</t>
         </is>
       </c>
       <c r="J521" t="inlineStr">
         <is>
-          <t>溶血性尿毒症综合征</t>
+          <t>贾第虫病</t>
         </is>
       </c>
       <c r="K521" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Parasitic</t>
         </is>
       </c>
       <c r="L521" t="inlineStr">
@@ -75496,17 +75496,17 @@
         </is>
       </c>
       <c r="N521" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="O521" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="R521" t="n">
-        <v>0.001195539327995473</v>
+        <v>0.05738588774378273</v>
       </c>
       <c r="U521" t="inlineStr">
         <is>
-          <t>HOLD_DE_a61a288370164339f3a7983800cd</t>
+          <t>HOLD_DE_e5f12cc63c1550ced86113ed9668</t>
         </is>
       </c>
       <c r="AA521" t="inlineStr">
@@ -75526,7 +75526,7 @@
       </c>
       <c r="AS521" t="inlineStr">
         <is>
-          <t>HOLD_DE_a61a288370164339f3a7983800cd</t>
+          <t>HOLD_DE_e5f12cc63c1550ced86113ed9668</t>
         </is>
       </c>
       <c r="AT521" t="n">
@@ -75611,22 +75611,22 @@
       </c>
       <c r="H522" t="inlineStr">
         <is>
-          <t>D105</t>
+          <t>D102</t>
         </is>
       </c>
       <c r="I522" t="inlineStr">
         <is>
-          <t>Shigellosis</t>
+          <t>Hantavirus infection</t>
         </is>
       </c>
       <c r="J522" t="inlineStr">
         <is>
-          <t>志贺菌病</t>
+          <t>汉坦病毒感染</t>
         </is>
       </c>
       <c r="K522" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L522" t="inlineStr">
@@ -75640,17 +75640,17 @@
         </is>
       </c>
       <c r="N522" t="n">
-        <v>93</v>
+        <v>4</v>
       </c>
       <c r="O522" t="n">
-        <v>93</v>
+        <v>4</v>
       </c>
       <c r="R522" t="n">
-        <v>0.111185157503579</v>
+        <v>0.004782157311981893</v>
       </c>
       <c r="U522" t="inlineStr">
         <is>
-          <t>HOLD_DE_295316a229986b9959d2b9e07dab</t>
+          <t>HOLD_DE_5cd9254a79f73f7e76719209af51</t>
         </is>
       </c>
       <c r="AA522" t="inlineStr">
@@ -75670,7 +75670,7 @@
       </c>
       <c r="AS522" t="inlineStr">
         <is>
-          <t>HOLD_DE_295316a229986b9959d2b9e07dab</t>
+          <t>HOLD_DE_5cd9254a79f73f7e76719209af51</t>
         </is>
       </c>
       <c r="AT522" t="n">
@@ -75755,17 +75755,17 @@
       </c>
       <c r="H523" t="inlineStr">
         <is>
-          <t>D106</t>
+          <t>D103</t>
         </is>
       </c>
       <c r="I523" t="inlineStr">
         <is>
-          <t>Invasive pneumococcal disease</t>
+          <t>Hemolytic uremic syndrome</t>
         </is>
       </c>
       <c r="J523" t="inlineStr">
         <is>
-          <t>侵袭性肺炎球菌病</t>
+          <t>溶血性尿毒症综合征</t>
         </is>
       </c>
       <c r="K523" t="inlineStr">
@@ -75784,17 +75784,17 @@
         </is>
       </c>
       <c r="N523" t="n">
-        <v>165</v>
+        <v>1</v>
       </c>
       <c r="O523" t="n">
-        <v>165</v>
+        <v>1</v>
       </c>
       <c r="R523" t="n">
-        <v>0.1972639891192531</v>
+        <v>0.001195539327995473</v>
       </c>
       <c r="U523" t="inlineStr">
         <is>
-          <t>HOLD_DE_86c6a86499a31ba0f180631d65d1</t>
+          <t>HOLD_DE_a61a288370164339f3a7983800cd</t>
         </is>
       </c>
       <c r="AA523" t="inlineStr">
@@ -75814,7 +75814,7 @@
       </c>
       <c r="AS523" t="inlineStr">
         <is>
-          <t>HOLD_DE_86c6a86499a31ba0f180631d65d1</t>
+          <t>HOLD_DE_a61a288370164339f3a7983800cd</t>
         </is>
       </c>
       <c r="AT523" t="n">
@@ -75899,17 +75899,17 @@
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D105</t>
         </is>
       </c>
       <c r="I524" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Shigellosis</t>
         </is>
       </c>
       <c r="J524" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>志贺菌病</t>
         </is>
       </c>
       <c r="K524" t="inlineStr">
@@ -75928,17 +75928,17 @@
         </is>
       </c>
       <c r="N524" t="n">
-        <v>63</v>
+        <v>96</v>
       </c>
       <c r="O524" t="n">
-        <v>63</v>
+        <v>96</v>
       </c>
       <c r="R524" t="n">
-        <v>0.07531897766371483</v>
+        <v>0.1147717754875655</v>
       </c>
       <c r="U524" t="inlineStr">
         <is>
-          <t>HOLD_DE_d79d74d6e3f0785d9f599cb1b651</t>
+          <t>HOLD_DE_295316a229986b9959d2b9e07dab</t>
         </is>
       </c>
       <c r="AA524" t="inlineStr">
@@ -75958,7 +75958,7 @@
       </c>
       <c r="AS524" t="inlineStr">
         <is>
-          <t>HOLD_DE_d79d74d6e3f0785d9f599cb1b651</t>
+          <t>HOLD_DE_295316a229986b9959d2b9e07dab</t>
         </is>
       </c>
       <c r="AT524" t="n">
@@ -76043,17 +76043,17 @@
       </c>
       <c r="H525" t="inlineStr">
         <is>
-          <t>D108</t>
+          <t>D106</t>
         </is>
       </c>
       <c r="I525" t="inlineStr">
         <is>
-          <t>Listeriosis</t>
+          <t>Invasive pneumococcal disease</t>
         </is>
       </c>
       <c r="J525" t="inlineStr">
         <is>
-          <t>李斯特菌病</t>
+          <t>侵袭性肺炎球菌病</t>
         </is>
       </c>
       <c r="K525" t="inlineStr">
@@ -76072,17 +76072,17 @@
         </is>
       </c>
       <c r="N525" t="n">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="O525" t="n">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="R525" t="n">
-        <v>0.01434647193594568</v>
+        <v>0.1960684497912576</v>
       </c>
       <c r="U525" t="inlineStr">
         <is>
-          <t>HOLD_DE_bcf77dd5c39d1691d1b7e1b96a96</t>
+          <t>HOLD_DE_86c6a86499a31ba0f180631d65d1</t>
         </is>
       </c>
       <c r="AA525" t="inlineStr">
@@ -76102,7 +76102,7 @@
       </c>
       <c r="AS525" t="inlineStr">
         <is>
-          <t>HOLD_DE_bcf77dd5c39d1691d1b7e1b96a96</t>
+          <t>HOLD_DE_86c6a86499a31ba0f180631d65d1</t>
         </is>
       </c>
       <c r="AT525" t="n">
@@ -76187,17 +76187,17 @@
       </c>
       <c r="H526" t="inlineStr">
         <is>
-          <t>D109</t>
+          <t>D107</t>
         </is>
       </c>
       <c r="I526" t="inlineStr">
         <is>
-          <t>Lyme disease</t>
+          <t>Legionellosis</t>
         </is>
       </c>
       <c r="J526" t="inlineStr">
         <is>
-          <t>莱姆病</t>
+          <t>军团菌病</t>
         </is>
       </c>
       <c r="K526" t="inlineStr">
@@ -76216,17 +76216,17 @@
         </is>
       </c>
       <c r="N526" t="n">
-        <v>182</v>
+        <v>64</v>
       </c>
       <c r="O526" t="n">
-        <v>182</v>
+        <v>64</v>
       </c>
       <c r="R526" t="n">
-        <v>0.2175881576951762</v>
+        <v>0.07651451699171029</v>
       </c>
       <c r="U526" t="inlineStr">
         <is>
-          <t>HOLD_DE_b250db3ee9361ea08d0baa333747</t>
+          <t>HOLD_DE_d79d74d6e3f0785d9f599cb1b651</t>
         </is>
       </c>
       <c r="AA526" t="inlineStr">
@@ -76246,7 +76246,7 @@
       </c>
       <c r="AS526" t="inlineStr">
         <is>
-          <t>HOLD_DE_b250db3ee9361ea08d0baa333747</t>
+          <t>HOLD_DE_d79d74d6e3f0785d9f599cb1b651</t>
         </is>
       </c>
       <c r="AT526" t="n">
@@ -76331,17 +76331,17 @@
       </c>
       <c r="H527" t="inlineStr">
         <is>
-          <t>D110</t>
+          <t>D108</t>
         </is>
       </c>
       <c r="I527" t="inlineStr">
         <is>
-          <t>Meningococcal disease</t>
+          <t>Listeriosis</t>
         </is>
       </c>
       <c r="J527" t="inlineStr">
         <is>
-          <t>脑膜炎球菌病</t>
+          <t>李斯特菌病</t>
         </is>
       </c>
       <c r="K527" t="inlineStr">
@@ -76360,17 +76360,17 @@
         </is>
       </c>
       <c r="N527" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="O527" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="R527" t="n">
-        <v>0.00358661798398642</v>
+        <v>0.01434647193594568</v>
       </c>
       <c r="U527" t="inlineStr">
         <is>
-          <t>HOLD_DE_e9bcf1404b2e1bd6b7512d0fe790</t>
+          <t>HOLD_DE_bcf77dd5c39d1691d1b7e1b96a96</t>
         </is>
       </c>
       <c r="AA527" t="inlineStr">
@@ -76390,7 +76390,7 @@
       </c>
       <c r="AS527" t="inlineStr">
         <is>
-          <t>HOLD_DE_e9bcf1404b2e1bd6b7512d0fe790</t>
+          <t>HOLD_DE_bcf77dd5c39d1691d1b7e1b96a96</t>
         </is>
       </c>
       <c r="AT527" t="n">
@@ -76475,17 +76475,17 @@
       </c>
       <c r="H528" t="inlineStr">
         <is>
-          <t>D113</t>
+          <t>D109</t>
         </is>
       </c>
       <c r="I528" t="inlineStr">
         <is>
-          <t>Q fever</t>
+          <t>Lyme disease</t>
         </is>
       </c>
       <c r="J528" t="inlineStr">
         <is>
-          <t>Q热</t>
+          <t>莱姆病</t>
         </is>
       </c>
       <c r="K528" t="inlineStr">
@@ -76504,17 +76504,17 @@
         </is>
       </c>
       <c r="N528" t="n">
-        <v>2</v>
+        <v>183</v>
       </c>
       <c r="O528" t="n">
-        <v>2</v>
+        <v>183</v>
       </c>
       <c r="R528" t="n">
-        <v>0.002391078655990946</v>
+        <v>0.2187836970231716</v>
       </c>
       <c r="U528" t="inlineStr">
         <is>
-          <t>HOLD_DE_4ea6e71b5e9b20f8d58a1d7a049f</t>
+          <t>HOLD_DE_b250db3ee9361ea08d0baa333747</t>
         </is>
       </c>
       <c r="AA528" t="inlineStr">
@@ -76534,7 +76534,7 @@
       </c>
       <c r="AS528" t="inlineStr">
         <is>
-          <t>HOLD_DE_4ea6e71b5e9b20f8d58a1d7a049f</t>
+          <t>HOLD_DE_b250db3ee9361ea08d0baa333747</t>
         </is>
       </c>
       <c r="AT528" t="n">
@@ -76619,17 +76619,17 @@
       </c>
       <c r="H529" t="inlineStr">
         <is>
-          <t>D114</t>
+          <t>D110</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>Salmonellosis</t>
+          <t>Meningococcal disease</t>
         </is>
       </c>
       <c r="J529" t="inlineStr">
         <is>
-          <t>沙门氏菌病</t>
+          <t>脑膜炎球菌病</t>
         </is>
       </c>
       <c r="K529" t="inlineStr">
@@ -76648,17 +76648,17 @@
         </is>
       </c>
       <c r="N529" t="n">
-        <v>244</v>
+        <v>3</v>
       </c>
       <c r="O529" t="n">
-        <v>244</v>
+        <v>3</v>
       </c>
       <c r="R529" t="n">
-        <v>0.2917115960308955</v>
+        <v>0.00358661798398642</v>
       </c>
       <c r="U529" t="inlineStr">
         <is>
-          <t>HOLD_DE_b577741583987e73a68c7b256222</t>
+          <t>HOLD_DE_e9bcf1404b2e1bd6b7512d0fe790</t>
         </is>
       </c>
       <c r="AA529" t="inlineStr">
@@ -76678,7 +76678,7 @@
       </c>
       <c r="AS529" t="inlineStr">
         <is>
-          <t>HOLD_DE_b577741583987e73a68c7b256222</t>
+          <t>HOLD_DE_e9bcf1404b2e1bd6b7512d0fe790</t>
         </is>
       </c>
       <c r="AT529" t="n">
@@ -76763,17 +76763,17 @@
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>D115</t>
+          <t>D113</t>
         </is>
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>Shiga toxin-producing Escherichia coli infection</t>
+          <t>Q fever</t>
         </is>
       </c>
       <c r="J530" t="inlineStr">
         <is>
-          <t>产志贺毒素大肠杆菌感染</t>
+          <t>Q热</t>
         </is>
       </c>
       <c r="K530" t="inlineStr">
@@ -76792,17 +76792,17 @@
         </is>
       </c>
       <c r="N530" t="n">
-        <v>136</v>
+        <v>2</v>
       </c>
       <c r="O530" t="n">
-        <v>136</v>
+        <v>2</v>
       </c>
       <c r="R530" t="n">
-        <v>0.1625933486073844</v>
+        <v>0.002391078655990946</v>
       </c>
       <c r="U530" t="inlineStr">
         <is>
-          <t>HOLD_DE_059854ba4ccf7917ff23b547178c</t>
+          <t>HOLD_DE_4ea6e71b5e9b20f8d58a1d7a049f</t>
         </is>
       </c>
       <c r="AA530" t="inlineStr">
@@ -76822,7 +76822,7 @@
       </c>
       <c r="AS530" t="inlineStr">
         <is>
-          <t>HOLD_DE_059854ba4ccf7917ff23b547178c</t>
+          <t>HOLD_DE_4ea6e71b5e9b20f8d58a1d7a049f</t>
         </is>
       </c>
       <c r="AT530" t="n">
@@ -76907,17 +76907,17 @@
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>D124</t>
+          <t>D114</t>
         </is>
       </c>
       <c r="I531" t="inlineStr">
         <is>
-          <t>Typhoid fever</t>
+          <t>Salmonellosis</t>
         </is>
       </c>
       <c r="J531" t="inlineStr">
         <is>
-          <t>伤寒</t>
+          <t>沙门氏菌病</t>
         </is>
       </c>
       <c r="K531" t="inlineStr">
@@ -76936,17 +76936,17 @@
         </is>
       </c>
       <c r="N531" t="n">
-        <v>1</v>
+        <v>260</v>
       </c>
       <c r="O531" t="n">
-        <v>1</v>
+        <v>260</v>
       </c>
       <c r="R531" t="n">
-        <v>0.001195539327995473</v>
+        <v>0.3108402252788231</v>
       </c>
       <c r="U531" t="inlineStr">
         <is>
-          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
+          <t>HOLD_DE_b577741583987e73a68c7b256222</t>
         </is>
       </c>
       <c r="AA531" t="inlineStr">
@@ -76966,7 +76966,7 @@
       </c>
       <c r="AS531" t="inlineStr">
         <is>
-          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
+          <t>HOLD_DE_b577741583987e73a68c7b256222</t>
         </is>
       </c>
       <c r="AT531" t="n">
@@ -77051,17 +77051,17 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>D126</t>
+          <t>D115</t>
         </is>
       </c>
       <c r="I532" t="inlineStr">
         <is>
-          <t>Vibriosis</t>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
         </is>
       </c>
       <c r="J532" t="inlineStr">
         <is>
-          <t>弧菌病</t>
+          <t>产志贺毒素大肠杆菌感染</t>
         </is>
       </c>
       <c r="K532" t="inlineStr">
@@ -77080,17 +77080,17 @@
         </is>
       </c>
       <c r="N532" t="n">
-        <v>2</v>
+        <v>142</v>
       </c>
       <c r="O532" t="n">
-        <v>2</v>
+        <v>142</v>
       </c>
       <c r="R532" t="n">
-        <v>0.002391078655990946</v>
+        <v>0.1697665845753572</v>
       </c>
       <c r="U532" t="inlineStr">
         <is>
-          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
+          <t>HOLD_DE_059854ba4ccf7917ff23b547178c</t>
         </is>
       </c>
       <c r="AA532" t="inlineStr">
@@ -77110,7 +77110,7 @@
       </c>
       <c r="AS532" t="inlineStr">
         <is>
-          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
+          <t>HOLD_DE_059854ba4ccf7917ff23b547178c</t>
         </is>
       </c>
       <c r="AT532" t="n">
@@ -77195,22 +77195,22 @@
       </c>
       <c r="H533" t="inlineStr">
         <is>
-          <t>D142</t>
+          <t>D123</t>
         </is>
       </c>
       <c r="I533" t="inlineStr">
         <is>
-          <t>Respiratory syncytial virus infection (RSV)</t>
+          <t>Tularemia</t>
         </is>
       </c>
       <c r="J533" t="inlineStr">
         <is>
-          <t>呼吸道合胞病毒感染</t>
+          <t>土拉菌病</t>
         </is>
       </c>
       <c r="K533" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L533" t="inlineStr">
@@ -77224,17 +77224,17 @@
         </is>
       </c>
       <c r="N533" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="O533" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="R533" t="n">
-        <v>0.04423495513583252</v>
+        <v>0.01195539327995473</v>
       </c>
       <c r="U533" t="inlineStr">
         <is>
-          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
+          <t>HOLD_DE_b849fa63b7ae6fabb95bdf916fe8</t>
         </is>
       </c>
       <c r="AA533" t="inlineStr">
@@ -77254,7 +77254,7 @@
       </c>
       <c r="AS533" t="inlineStr">
         <is>
-          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
+          <t>HOLD_DE_b849fa63b7ae6fabb95bdf916fe8</t>
         </is>
       </c>
       <c r="AT533" t="n">
@@ -77339,17 +77339,17 @@
       </c>
       <c r="H534" t="inlineStr">
         <is>
-          <t>D155</t>
+          <t>D124</t>
         </is>
       </c>
       <c r="I534" t="inlineStr">
         <is>
-          <t>Yersiniosis</t>
+          <t>Typhoid fever</t>
         </is>
       </c>
       <c r="J534" t="inlineStr">
         <is>
-          <t>耶尔森菌病</t>
+          <t>伤寒</t>
         </is>
       </c>
       <c r="K534" t="inlineStr">
@@ -77368,17 +77368,17 @@
         </is>
       </c>
       <c r="N534" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="O534" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="R534" t="n">
-        <v>0.04543049446382799</v>
+        <v>0.001195539327995473</v>
       </c>
       <c r="U534" t="inlineStr">
         <is>
-          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
+          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
         </is>
       </c>
       <c r="AA534" t="inlineStr">
@@ -77398,7 +77398,7 @@
       </c>
       <c r="AS534" t="inlineStr">
         <is>
-          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
+          <t>HOLD_DE_cd1ba4c777ff5793402d1adae771</t>
         </is>
       </c>
       <c r="AT534" t="n">
@@ -77483,22 +77483,22 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>D199</t>
+          <t>D126</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
         <is>
-          <t>Rotavirus infection</t>
+          <t>Vibriosis</t>
         </is>
       </c>
       <c r="J535" t="inlineStr">
         <is>
-          <t>轮状病毒感染</t>
+          <t>弧菌病</t>
         </is>
       </c>
       <c r="K535" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L535" t="inlineStr">
@@ -77512,17 +77512,17 @@
         </is>
       </c>
       <c r="N535" t="n">
-        <v>153</v>
+        <v>2</v>
       </c>
       <c r="O535" t="n">
-        <v>153</v>
+        <v>2</v>
       </c>
       <c r="R535" t="n">
-        <v>0.1829175171833074</v>
+        <v>0.002391078655990946</v>
       </c>
       <c r="U535" t="inlineStr">
         <is>
-          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
+          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
         </is>
       </c>
       <c r="AA535" t="inlineStr">
@@ -77542,7 +77542,7 @@
       </c>
       <c r="AS535" t="inlineStr">
         <is>
-          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
+          <t>HOLD_DE_16f5df972f268cf6814c42ea1fa0</t>
         </is>
       </c>
       <c r="AT535" t="n">
@@ -77627,17 +77627,17 @@
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>D205</t>
+          <t>D142</t>
         </is>
       </c>
       <c r="I536" t="inlineStr">
         <is>
-          <t>Tick-borne encephalitis</t>
+          <t>Respiratory syncytial virus infection (RSV)</t>
         </is>
       </c>
       <c r="J536" t="inlineStr">
         <is>
-          <t>蜱传脑炎</t>
+          <t>呼吸道合胞病毒感染</t>
         </is>
       </c>
       <c r="K536" t="inlineStr">
@@ -77656,17 +77656,17 @@
         </is>
       </c>
       <c r="N536" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="O536" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="R536" t="n">
-        <v>0.009564314623963786</v>
+        <v>0.04423495513583252</v>
       </c>
       <c r="U536" t="inlineStr">
         <is>
-          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
+          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
         </is>
       </c>
       <c r="AA536" t="inlineStr">
@@ -77686,7 +77686,7 @@
       </c>
       <c r="AS536" t="inlineStr">
         <is>
-          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
+          <t>HOLD_DE_26519904c83fe8dc106484ae7d9c</t>
         </is>
       </c>
       <c r="AT536" t="n">
@@ -77771,17 +77771,17 @@
       </c>
       <c r="H537" t="inlineStr">
         <is>
-          <t>D227</t>
+          <t>D155</t>
         </is>
       </c>
       <c r="I537" t="inlineStr">
         <is>
-          <t>Carbapenem-resistant Enterobacterales infection</t>
+          <t>Yersiniosis</t>
         </is>
       </c>
       <c r="J537" t="inlineStr">
         <is>
-          <t>碳青霉烯耐药肠杆菌目细菌感染</t>
+          <t>耶尔森菌病</t>
         </is>
       </c>
       <c r="K537" t="inlineStr">
@@ -77800,17 +77800,17 @@
         </is>
       </c>
       <c r="N537" t="n">
-        <v>214</v>
+        <v>42</v>
       </c>
       <c r="O537" t="n">
-        <v>214</v>
+        <v>42</v>
       </c>
       <c r="R537" t="n">
-        <v>0.2558454161910313</v>
+        <v>0.05021265177580988</v>
       </c>
       <c r="U537" t="inlineStr">
         <is>
-          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
+          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
         </is>
       </c>
       <c r="AA537" t="inlineStr">
@@ -77830,7 +77830,7 @@
       </c>
       <c r="AS537" t="inlineStr">
         <is>
-          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
+          <t>HOLD_DE_f8a42d099ba513454344dfcd2d5b</t>
         </is>
       </c>
       <c r="AT537" t="n">
@@ -77915,22 +77915,22 @@
       </c>
       <c r="H538" t="inlineStr">
         <is>
-          <t>D236</t>
+          <t>D199</t>
         </is>
       </c>
       <c r="I538" t="inlineStr">
         <is>
-          <t>Methicillin-resistant Staphylococcus aureus (MRSA) surveillance</t>
+          <t>Rotavirus infection</t>
         </is>
       </c>
       <c r="J538" t="inlineStr">
         <is>
-          <t>耐甲氧西林金黄色葡萄球菌（MRSA）监测</t>
+          <t>轮状病毒感染</t>
         </is>
       </c>
       <c r="K538" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L538" t="inlineStr">
@@ -77944,17 +77944,17 @@
         </is>
       </c>
       <c r="N538" t="n">
-        <v>19</v>
+        <v>157</v>
       </c>
       <c r="O538" t="n">
-        <v>19</v>
+        <v>157</v>
       </c>
       <c r="R538" t="n">
-        <v>0.022715247231914</v>
+        <v>0.1876996744952893</v>
       </c>
       <c r="U538" t="inlineStr">
         <is>
-          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
+          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
         </is>
       </c>
       <c r="AA538" t="inlineStr">
@@ -77974,7 +77974,7 @@
       </c>
       <c r="AS538" t="inlineStr">
         <is>
-          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
+          <t>HOLD_DE_52a585aee0ab7be71a4aa362be02</t>
         </is>
       </c>
       <c r="AT538" t="n">
@@ -78016,6 +78016,438 @@
         </is>
       </c>
       <c r="BC538" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>D205</t>
+        </is>
+      </c>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>Tick-borne encephalitis</t>
+        </is>
+      </c>
+      <c r="J539" t="inlineStr">
+        <is>
+          <t>蜱传脑炎</t>
+        </is>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L539" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="M539" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="N539" t="n">
+        <v>8</v>
+      </c>
+      <c r="O539" t="n">
+        <v>8</v>
+      </c>
+      <c r="R539" t="n">
+        <v>0.009564314623963786</v>
+      </c>
+      <c r="U539" t="inlineStr">
+        <is>
+          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
+        </is>
+      </c>
+      <c r="AA539" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AO539" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP539" t="inlineStr">
+        <is>
+          <t>published_series</t>
+        </is>
+      </c>
+      <c r="AS539" t="inlineStr">
+        <is>
+          <t>HOLD_DE_e35abc87a6dbbcbd594d5232c594</t>
+        </is>
+      </c>
+      <c r="AT539" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV539" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW539" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX539" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY539" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ539" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA539" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB539" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC539" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>D227</t>
+        </is>
+      </c>
+      <c r="I540" t="inlineStr">
+        <is>
+          <t>Carbapenem-resistant Enterobacterales infection</t>
+        </is>
+      </c>
+      <c r="J540" t="inlineStr">
+        <is>
+          <t>碳青霉烯耐药肠杆菌目细菌感染</t>
+        </is>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L540" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="M540" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="N540" t="n">
+        <v>217</v>
+      </c>
+      <c r="O540" t="n">
+        <v>217</v>
+      </c>
+      <c r="R540" t="n">
+        <v>0.2594320341750177</v>
+      </c>
+      <c r="U540" t="inlineStr">
+        <is>
+          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
+        </is>
+      </c>
+      <c r="AA540" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AO540" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP540" t="inlineStr">
+        <is>
+          <t>published_series</t>
+        </is>
+      </c>
+      <c r="AS540" t="inlineStr">
+        <is>
+          <t>HOLD_DE_3059f17f5d9a83da53708e7a0f25</t>
+        </is>
+      </c>
+      <c r="AT540" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV540" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW540" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX540" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY540" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ540" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA540" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB540" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC540" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>D236</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>Methicillin-resistant Staphylococcus aureus (MRSA) surveillance</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>耐甲氧西林金黄色葡萄球菌（MRSA）监测</t>
+        </is>
+      </c>
+      <c r="K541" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L541" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="M541" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="N541" t="n">
+        <v>19</v>
+      </c>
+      <c r="O541" t="n">
+        <v>19</v>
+      </c>
+      <c r="R541" t="n">
+        <v>0.022715247231914</v>
+      </c>
+      <c r="U541" t="inlineStr">
+        <is>
+          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
+        </is>
+      </c>
+      <c r="AA541" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AO541" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP541" t="inlineStr">
+        <is>
+          <t>published_series</t>
+        </is>
+      </c>
+      <c r="AS541" t="inlineStr">
+        <is>
+          <t>HOLD_DE_6ea32e254214cab9f62091fadbc0</t>
+        </is>
+      </c>
+      <c r="AT541" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV541" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="AW541" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="AX541" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="AY541" t="inlineStr">
+        <is>
+          <t>official_webforms_csv_export</t>
+        </is>
+      </c>
+      <c r="AZ541" t="inlineStr">
+        <is>
+          <t>rki_survstat</t>
+        </is>
+      </c>
+      <c r="BA541" t="inlineStr">
+        <is>
+          <t>Germany RKI SurvStat 2.0</t>
+        </is>
+      </c>
+      <c r="BB541" t="inlineStr">
+        <is>
+          <t>https://survstat.rki.de/Content/Query/Create.aspx</t>
+        </is>
+      </c>
+      <c r="BC541" t="inlineStr">
         <is>
           <t>official_webforms_csv_export</t>
         </is>
@@ -78137,7 +78569,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="10">
@@ -78147,7 +78579,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="11">
@@ -78199,7 +78631,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>61441</v>
+        <v>61660</v>
       </c>
     </row>
     <row r="16">

</xml_diff>